<commit_message>
Publica dashboard de agentes Copilot
</commit_message>
<xml_diff>
--- a/data/catalogo-agentes-operacionais-copilot.xlsx
+++ b/data/catalogo-agentes-operacionais-copilot.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalogo de agentes" sheetId="1" r:id="Rf9f2ddd906524653"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top 40 demos" sheetId="2" r:id="R19136d20214a41f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cowork playbook" sheetId="3" r:id="R184b8bb86a8945e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fontes" sheetId="4" r:id="R2b70e9082d164334"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Como escolher" sheetId="5" r:id="Re3753fef95d7478e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="6" r:id="Rb1d2ae9ebdf34d1e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalogo de agentes" sheetId="1" r:id="R74af03ca2194480c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top 40 demos" sheetId="2" r:id="R6c1066e5a3fe4416"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cowork playbook" sheetId="3" r:id="R21eed9f940094626"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fontes" sheetId="4" r:id="R4c2160cd1ff749cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Como escolher" sheetId="5" r:id="R1a3a3528c5bf4a40"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="6" r:id="Rff765057d3a94275"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -367,7 +367,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R70c7567a16ae4cbc"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re6a182a4fb68499d"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -397,7 +397,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rba51b45c0ad6495a"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2d7533e3d8684e72"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -18718,7 +18718,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7555c49157884b92"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0cb36700d14945ec"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20282,7 +20282,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7fa94b6e09c040c6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1900a96b372d4bb1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21028,7 +21028,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff9d9a634dda4eb2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5989c0bf6d0f4a2f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21592,7 +21592,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb6d717f19d547ec"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f0aa19c2d184749"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21736,7 +21736,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R287c545140fd407b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d1f51535f204a45"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22363,6 +22363,6 @@
     <x:mergeCell ref="A1:H1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda6789cc82f343be"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8feffe0995b84fbb"/>
 </x:worksheet>
 </file>
</xml_diff>